<commit_message>
added more validation data for inflow
</commit_message>
<xml_diff>
--- a/inflow_validation.xlsx
+++ b/inflow_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marita/Documents/GitHub/MFA2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2B579E-E15B-C34B-B5A1-C67F0E063856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE09FDB-9EBC-0045-80C5-77FB5B460E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="500" windowWidth="28800" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="15320" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tabla-6150" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="248">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -729,13 +729,61 @@
   </si>
   <si>
     <t>SOURCE2</t>
+  </si>
+  <si>
+    <t>ine</t>
+  </si>
+  <si>
+    <t>source 2</t>
+  </si>
+  <si>
+    <t>source 1</t>
+  </si>
+  <si>
+    <t>paper thomas sent</t>
+  </si>
+  <si>
+    <t>source 3</t>
+  </si>
+  <si>
+    <t>SOURCE3</t>
+  </si>
+  <si>
+    <t>https://www.bde.es/webbe/en/estadisticas/otras-clasificaciones/publicaciones/boletin-estadistico/capitulo-23.html</t>
+  </si>
+  <si>
+    <t>SOURCE4</t>
+  </si>
+  <si>
+    <t>source 4</t>
+  </si>
+  <si>
+    <t>https://www.funcas.es/wp-content/uploads/Migracion/Articulos/FUNCAS_PEE/010art14.pdf</t>
+  </si>
+  <si>
+    <t>SOURCE5</t>
+  </si>
+  <si>
+    <t>source 5</t>
+  </si>
+  <si>
+    <t>https://habitat.aq.upm.es/in/a003/ab003.html</t>
+  </si>
+  <si>
+    <t>SOURCE6</t>
+  </si>
+  <si>
+    <t>source 6</t>
+  </si>
+  <si>
+    <t>https://www.coam.org/media/Default%20Files/fundacion/biblioteca/revista-arquitectura-100/1959-1973/docs/revista-articulos/revista-arquitectura-1964-n66-pag58-62.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -748,11 +796,32 @@
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color indexed="8"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -788,13 +857,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -804,6 +873,11 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -825,16 +899,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1219200</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>1240367</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
+      <xdr:rowOff>160866</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>63058</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>105834</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>39774</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -863,8 +937,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11620500" y="406400"/>
-          <a:ext cx="7785100" cy="4419158"/>
+          <a:off x="19121967" y="533399"/>
+          <a:ext cx="7806267" cy="4349308"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1193,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F229"/>
+  <dimension ref="A1:M229"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39" style="1" customWidth="1"/>
@@ -1201,7 +1275,7 @@
     <col min="3" max="227" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1215,8 +1289,20 @@
       <c r="F1" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H1" t="s">
+        <v>239</v>
+      </c>
+      <c r="I1" t="s">
+        <v>242</v>
+      </c>
+      <c r="J1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1230,8 +1316,13 @@
         <f>SUM(B2:B13)</f>
         <v>155910</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F2" s="7"/>
+      <c r="G2" s="8">
+        <v>88254</v>
+      </c>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1245,8 +1336,13 @@
         <f>SUM(B14:B25)</f>
         <v>134338</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F3" s="7"/>
+      <c r="G3" s="8">
+        <v>97837</v>
+      </c>
+      <c r="H3" s="7"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -1260,8 +1356,13 @@
         <f>SUM(B26:B37)</f>
         <v>109481</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F4" s="7"/>
+      <c r="G4" s="8">
+        <v>87565</v>
+      </c>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
@@ -1275,8 +1376,13 @@
         <f>SUM(B38:B49)</f>
         <v>116458</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F5" s="7"/>
+      <c r="G5" s="8">
+        <v>89107</v>
+      </c>
+      <c r="H5" s="7"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -1290,8 +1396,13 @@
         <f>SUM(B50:B61)</f>
         <v>114030</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F6" s="7"/>
+      <c r="G6" s="8">
+        <v>91390</v>
+      </c>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -1305,8 +1416,13 @@
         <f>SUM(B62:B73)</f>
         <v>83561</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F7" s="7"/>
+      <c r="G7" s="8">
+        <v>85945</v>
+      </c>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1320,8 +1436,13 @@
         <f>SUM(B74:B85)</f>
         <v>92946</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F8" s="7"/>
+      <c r="G8" s="8">
+        <v>78789</v>
+      </c>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -1335,8 +1456,13 @@
         <f>SUM(B86:B97)</f>
         <v>91716</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F9" s="7"/>
+      <c r="G9" s="8">
+        <v>64354</v>
+      </c>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -1350,8 +1476,13 @@
         <f>SUM(B98:B109)</f>
         <v>83240</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="7"/>
+      <c r="G10" s="8">
+        <v>54610</v>
+      </c>
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
@@ -1365,8 +1496,13 @@
         <f>SUM(B110:B121)</f>
         <v>75134</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F11" s="7"/>
+      <c r="G11" s="8">
+        <v>40119</v>
+      </c>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1380,8 +1516,13 @@
         <f>SUM(B122:B133)</f>
         <v>76954</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F12" s="7"/>
+      <c r="G12" s="8">
+        <v>45152</v>
+      </c>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
@@ -1395,8 +1536,13 @@
         <f>SUM(B134:B145)</f>
         <v>117519</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F13" s="7"/>
+      <c r="G13" s="8">
+        <v>46822</v>
+      </c>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1410,8 +1556,13 @@
         <f>SUM(B146:B157)</f>
         <v>143771</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F14" s="7"/>
+      <c r="G14" s="8">
+        <v>64817</v>
+      </c>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1425,8 +1576,13 @@
         <f>SUM(B158:B169)</f>
         <v>155890</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F15" s="7"/>
+      <c r="G15" s="8">
+        <v>114991</v>
+      </c>
+      <c r="H15" s="9"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -1440,11 +1596,15 @@
         <f>SUM(B170:B181)</f>
         <v>174299</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="7">
         <v>80000</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G16" s="8">
+        <v>157405</v>
+      </c>
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -1458,11 +1618,15 @@
         <f>SUM(B182:B193)</f>
         <v>220612</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="7">
         <v>90000</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G17" s="8">
+        <v>240920</v>
+      </c>
+      <c r="H17" s="10"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1476,11 +1640,15 @@
         <f>SUM(B194:B205)</f>
         <v>218775</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="7">
         <v>110000</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G18" s="8">
+        <v>366887</v>
+      </c>
+      <c r="H18" s="10"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -1494,11 +1662,15 @@
         <f>SUM(B206:B217)</f>
         <v>278034</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="7">
         <v>260000</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G19" s="8">
+        <v>615072</v>
+      </c>
+      <c r="H19" s="10"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -1512,11 +1684,15 @@
         <f>SUM(B218:B229)</f>
         <v>326382</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="7">
         <v>650000</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G20" s="8">
+        <v>641419</v>
+      </c>
+      <c r="H20" s="10"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1526,11 +1702,15 @@
       <c r="D21">
         <v>2006</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="7">
         <v>850000</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G21" s="8">
+        <v>585584</v>
+      </c>
+      <c r="H21" s="10"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -1540,11 +1720,15 @@
       <c r="D22">
         <v>2005</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="7">
         <v>720000</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G22" s="8">
+        <v>524479</v>
+      </c>
+      <c r="H22" s="11"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -1554,11 +1738,15 @@
       <c r="D23">
         <v>2004</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="7">
         <v>680000</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G23" s="8">
+        <v>496785</v>
+      </c>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -1568,11 +1756,15 @@
       <c r="D24">
         <v>2003</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="7">
         <v>650000</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G24" s="8">
+        <v>458683</v>
+      </c>
+      <c r="H24" s="7"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -1582,11 +1774,15 @@
       <c r="D25">
         <v>2002</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="7">
         <v>520000</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G25" s="8">
+        <v>416683</v>
+      </c>
+      <c r="H25" s="7"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
@@ -1596,11 +1792,15 @@
       <c r="D26">
         <v>2001</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="7">
         <v>500000</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G26" s="8">
+        <v>365663</v>
+      </c>
+      <c r="H26" s="7"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>26</v>
       </c>
@@ -1610,11 +1810,15 @@
       <c r="D27">
         <v>2000</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="7">
         <v>530000</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G27" s="8">
+        <v>366776</v>
+      </c>
+      <c r="H27" s="7"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
@@ -1624,11 +1828,21 @@
       <c r="D28">
         <v>1999</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="7">
         <v>510000</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G28" s="8">
+        <v>321177</v>
+      </c>
+      <c r="H28" s="7"/>
+      <c r="L28" t="s">
+        <v>234</v>
+      </c>
+      <c r="M28" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
@@ -1638,11 +1852,21 @@
       <c r="D29">
         <v>1998</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="7">
         <v>440000</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G29" s="8">
+        <v>275596</v>
+      </c>
+      <c r="H29" s="7"/>
+      <c r="L29" t="s">
+        <v>233</v>
+      </c>
+      <c r="M29" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
@@ -1652,315 +1876,610 @@
       <c r="D30">
         <v>1997</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="7">
         <v>350000</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G30" s="8">
+        <v>272336</v>
+      </c>
+      <c r="H30" s="7"/>
+      <c r="L30" t="s">
+        <v>236</v>
+      </c>
+      <c r="M30" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="5">
         <v>8154</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D31">
+        <v>1996</v>
+      </c>
+      <c r="F31" s="7"/>
+      <c r="G31" s="8">
+        <v>253378</v>
+      </c>
+      <c r="H31" s="7"/>
+      <c r="L31" t="s">
+        <v>240</v>
+      </c>
+      <c r="M31" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="5">
         <v>10119</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <v>1995</v>
+      </c>
+      <c r="F32" s="7"/>
+      <c r="G32" s="8">
+        <v>242122</v>
+      </c>
+      <c r="H32" s="7"/>
+      <c r="L32" t="s">
+        <v>243</v>
+      </c>
+      <c r="M32" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B33" s="5">
         <v>10635</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <v>1994</v>
+      </c>
+      <c r="F33" s="7"/>
+      <c r="G33" s="8">
+        <v>219553</v>
+      </c>
+      <c r="H33" s="7"/>
+      <c r="L33" t="s">
+        <v>246</v>
+      </c>
+      <c r="M33" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B34" s="5">
         <v>8087</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <v>1993</v>
+      </c>
+      <c r="F34" s="7"/>
+      <c r="G34" s="8">
+        <v>205404</v>
+      </c>
+      <c r="H34" s="7"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B35" s="5">
         <v>10364</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <v>1992</v>
+      </c>
+      <c r="F35" s="7"/>
+      <c r="G35" s="8">
+        <v>205893</v>
+      </c>
+      <c r="H35" s="7"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>35</v>
       </c>
       <c r="B36" s="5">
         <v>9541</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <v>1991</v>
+      </c>
+      <c r="I36">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B37" s="5">
         <v>10571</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <v>1990</v>
+      </c>
+      <c r="I37">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B38" s="3">
         <v>7804</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <v>1989</v>
+      </c>
+      <c r="I38">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="3">
         <v>9978</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <v>1988</v>
+      </c>
+      <c r="I39">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B40" s="3">
         <v>8781</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <v>1987</v>
+      </c>
+      <c r="I40">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B41" s="3">
         <v>10181</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <v>1986</v>
+      </c>
+      <c r="I41">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B42" s="3">
         <v>10164</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D42">
+        <v>1985</v>
+      </c>
+      <c r="I42">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B43" s="3">
         <v>8924</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D43">
+        <v>1984</v>
+      </c>
+      <c r="I43">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B44" s="3">
         <v>9457</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D44">
+        <v>1983</v>
+      </c>
+      <c r="I44">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B45" s="3">
         <v>10242</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D45">
+        <v>1982</v>
+      </c>
+      <c r="I45">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B46" s="3">
         <v>8615</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D46">
+        <v>1981</v>
+      </c>
+      <c r="I46">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B47" s="3">
         <v>11317</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D47">
+        <v>1980</v>
+      </c>
+      <c r="I47">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B48" s="3">
         <v>10925</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D48">
+        <v>1979</v>
+      </c>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48">
+        <v>367083</v>
+      </c>
+      <c r="I48">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B49" s="3">
         <v>10070</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D49">
+        <v>1978</v>
+      </c>
+      <c r="H49">
+        <v>348645</v>
+      </c>
+      <c r="I49">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>49</v>
       </c>
       <c r="B50" s="5">
         <v>9543</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D50">
+        <v>1977</v>
+      </c>
+      <c r="H50">
+        <v>406071</v>
+      </c>
+      <c r="I50">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>50</v>
       </c>
       <c r="B51" s="5">
         <v>10243</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D51">
+        <v>1976</v>
+      </c>
+      <c r="H51">
+        <v>376038</v>
+      </c>
+      <c r="I51">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B52" s="5">
         <v>9349</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D52">
+        <v>1975</v>
+      </c>
+      <c r="H52">
+        <v>388779</v>
+      </c>
+      <c r="I52">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B53" s="5">
         <v>10909</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D53">
+        <v>1974</v>
+      </c>
+      <c r="H53">
+        <v>568834</v>
+      </c>
+      <c r="I53">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B54" s="5">
         <v>9536</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D54">
+        <v>1973</v>
+      </c>
+      <c r="H54">
+        <v>696446</v>
+      </c>
+      <c r="I54">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B55" s="5">
         <v>9262</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D55">
+        <v>1972</v>
+      </c>
+      <c r="H55">
+        <v>598065</v>
+      </c>
+      <c r="I55">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B56" s="5">
         <v>9167</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D56">
+        <v>1971</v>
+      </c>
+      <c r="H56">
+        <v>357658</v>
+      </c>
+      <c r="I56">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B57" s="5">
         <v>9044</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D57">
+        <v>1970</v>
+      </c>
+      <c r="H57">
+        <v>349995</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B58" s="5">
         <v>8501</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D58">
+        <v>1960</v>
+      </c>
+      <c r="J58">
+        <v>128000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
         <v>58</v>
       </c>
       <c r="B59" s="5">
         <v>9949</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D59">
+        <v>1959</v>
+      </c>
+      <c r="J59">
+        <v>114000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>59</v>
       </c>
       <c r="B60" s="5">
         <v>10002</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D60">
+        <v>1958</v>
+      </c>
+      <c r="J60">
+        <v>101000</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>60</v>
       </c>
       <c r="B61" s="5">
         <v>8525</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D61">
+        <v>1957</v>
+      </c>
+      <c r="J61">
+        <v>98000</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B62" s="3">
         <v>7310</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D62">
+        <v>1956</v>
+      </c>
+      <c r="J62">
+        <v>121800</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B63" s="3">
         <v>7924</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D63">
+        <v>1955</v>
+      </c>
+      <c r="J63">
+        <v>112200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B64" s="3">
         <v>7682</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D64">
+        <v>1954</v>
+      </c>
+      <c r="J64">
+        <v>87200</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>64</v>
       </c>
       <c r="B65" s="3">
         <v>8404</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D65">
+        <v>1953</v>
+      </c>
+      <c r="J65">
+        <v>67200</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B66" s="3">
         <v>6818</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D66">
+        <v>1952</v>
+      </c>
+      <c r="J66">
+        <v>63300</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B67" s="3">
         <v>6783</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D67">
+        <v>1951</v>
+      </c>
+      <c r="J67">
+        <v>56500</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B68" s="3">
         <v>5474</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D68">
+        <v>1950</v>
+      </c>
+      <c r="J68">
+        <v>53400</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>68</v>
       </c>
@@ -1968,7 +2487,7 @@
         <v>4277</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>69</v>
       </c>
@@ -1976,7 +2495,7 @@
         <v>4676</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>70</v>
       </c>
@@ -1984,7 +2503,7 @@
         <v>6650</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>71</v>
       </c>
@@ -1992,7 +2511,7 @@
         <v>9116</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>72</v>
       </c>
@@ -2000,7 +2519,7 @@
         <v>8447</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
         <v>73</v>
       </c>
@@ -2008,7 +2527,7 @@
         <v>6557</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
         <v>74</v>
       </c>
@@ -2016,7 +2535,7 @@
         <v>7701</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
         <v>75</v>
       </c>
@@ -2024,7 +2543,7 @@
         <v>8103</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
         <v>76</v>
       </c>
@@ -2032,7 +2551,7 @@
         <v>6490</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
         <v>77</v>
       </c>
@@ -2040,7 +2559,7 @@
         <v>6359</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
         <v>78</v>
       </c>
@@ -2048,7 +2567,7 @@
         <v>8588</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
         <v>79</v>
       </c>

</xml_diff>

<commit_message>
added even more validation data
</commit_message>
<xml_diff>
--- a/inflow_validation.xlsx
+++ b/inflow_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marita/Documents/GitHub/MFA2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE09FDB-9EBC-0045-80C5-77FB5B460E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC3C3D92-751A-7C48-8F1A-EF8448178246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="15320" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tabla-6150" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="240">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -239,39 +239,6 @@
     <t>2020M06</t>
   </si>
   <si>
-    <t>2020M05</t>
-  </si>
-  <si>
-    <t>2020M04</t>
-  </si>
-  <si>
-    <t>2020M03</t>
-  </si>
-  <si>
-    <t>2020M02</t>
-  </si>
-  <si>
-    <t>2020M01</t>
-  </si>
-  <si>
-    <t>2019M12</t>
-  </si>
-  <si>
-    <t>2019M11</t>
-  </si>
-  <si>
-    <t>2019M10</t>
-  </si>
-  <si>
-    <t>2019M09</t>
-  </si>
-  <si>
-    <t>2019M08</t>
-  </si>
-  <si>
-    <t>2019M07</t>
-  </si>
-  <si>
     <t>2019M06</t>
   </si>
   <si>
@@ -777,13 +744,22 @@
   </si>
   <si>
     <t>https://www.coam.org/media/Default%20Files/fundacion/biblioteca/revista-arquitectura-100/1959-1973/docs/revista-articulos/revista-arquitectura-1964-n66-pag58-62.pdf</t>
+  </si>
+  <si>
+    <t>SOURCE7</t>
+  </si>
+  <si>
+    <t>source 7</t>
+  </si>
+  <si>
+    <t>demolition</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -823,6 +799,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -857,7 +840,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -873,11 +856,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -899,16 +881,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>1240367</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>160866</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>322403</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>105834</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>39774</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>678003</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>68294</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -937,8 +919,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19121967" y="533399"/>
-          <a:ext cx="7806267" cy="4349308"/>
+          <a:off x="21789859" y="0"/>
+          <a:ext cx="7763933" cy="4424171"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1267,42 +1249,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M229"/>
+  <dimension ref="A1:O229"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39" style="1" customWidth="1"/>
     <col min="2" max="2" width="19.5" style="1" customWidth="1"/>
-    <col min="3" max="227" width="19.5" customWidth="1"/>
+    <col min="3" max="3" width="19.5" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="5" max="227" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="D1" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="E1" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="F1" t="s">
+        <v>220</v>
+      </c>
+      <c r="G1" t="s">
+        <v>226</v>
+      </c>
+      <c r="H1" t="s">
+        <v>228</v>
+      </c>
+      <c r="I1" t="s">
         <v>231</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
+        <v>234</v>
+      </c>
+      <c r="K1" t="s">
         <v>237</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>239</v>
       </c>
-      <c r="I1" t="s">
-        <v>242</v>
-      </c>
-      <c r="J1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1316,13 +1306,13 @@
         <f>SUM(B2:B13)</f>
         <v>155910</v>
       </c>
-      <c r="F2" s="7"/>
-      <c r="G2" s="8">
+      <c r="F2" s="1"/>
+      <c r="G2" s="7">
         <v>88254</v>
       </c>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1336,13 +1326,13 @@
         <f>SUM(B14:B25)</f>
         <v>134338</v>
       </c>
-      <c r="F3" s="7"/>
-      <c r="G3" s="8">
+      <c r="F3" s="1"/>
+      <c r="G3" s="7">
         <v>97837</v>
       </c>
-      <c r="H3" s="7"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -1356,13 +1346,13 @@
         <f>SUM(B26:B37)</f>
         <v>109481</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="8">
+      <c r="F4" s="1"/>
+      <c r="G4" s="7">
         <v>87565</v>
       </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
@@ -1376,13 +1366,13 @@
         <f>SUM(B38:B49)</f>
         <v>116458</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="8">
+      <c r="F5" s="1"/>
+      <c r="G5" s="7">
         <v>89107</v>
       </c>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -1393,16 +1383,16 @@
         <v>2021</v>
       </c>
       <c r="E6" s="6">
-        <f>SUM(B50:B61)</f>
+        <f>SUM(B50:B72)</f>
         <v>114030</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="8">
+      <c r="F6" s="1"/>
+      <c r="G6" s="7">
         <v>91390</v>
       </c>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -1413,16 +1403,19 @@
         <v>2020</v>
       </c>
       <c r="E7" s="6">
-        <f>SUM(B62:B73)</f>
-        <v>83561</v>
-      </c>
-      <c r="F7" s="7"/>
-      <c r="G7" s="8">
+        <f>SUM(B69:B79)</f>
+        <v>87372</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="7">
         <v>85945</v>
       </c>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H7" s="1"/>
+      <c r="K7" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
@@ -1433,16 +1426,19 @@
         <v>2019</v>
       </c>
       <c r="E8" s="6">
-        <f>SUM(B74:B85)</f>
-        <v>92946</v>
-      </c>
-      <c r="F8" s="7"/>
-      <c r="G8" s="8">
+        <f>SUM(B80:B85)</f>
+        <v>49148</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="7">
         <v>78789</v>
       </c>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H8" s="1"/>
+      <c r="K8" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
@@ -1456,13 +1452,16 @@
         <f>SUM(B86:B97)</f>
         <v>91716</v>
       </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8">
+      <c r="F9" s="1"/>
+      <c r="G9" s="7">
         <v>64354</v>
       </c>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H9" s="1"/>
+      <c r="K9" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
@@ -1476,13 +1475,16 @@
         <f>SUM(B98:B109)</f>
         <v>83240</v>
       </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="8">
+      <c r="F10" s="1"/>
+      <c r="G10" s="7">
         <v>54610</v>
       </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H10" s="1"/>
+      <c r="K10" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
@@ -1496,13 +1498,16 @@
         <f>SUM(B110:B121)</f>
         <v>75134</v>
       </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="8">
+      <c r="F11" s="1"/>
+      <c r="G11" s="7">
         <v>40119</v>
       </c>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H11" s="1"/>
+      <c r="K11" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1516,13 +1521,16 @@
         <f>SUM(B122:B133)</f>
         <v>76954</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8">
+      <c r="F12" s="1"/>
+      <c r="G12" s="7">
         <v>45152</v>
       </c>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H12" s="1"/>
+      <c r="K12" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>12</v>
       </c>
@@ -1536,13 +1544,16 @@
         <f>SUM(B134:B145)</f>
         <v>117519</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="8">
+      <c r="F13" s="1"/>
+      <c r="G13" s="7">
         <v>46822</v>
       </c>
-      <c r="H13" s="7"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H13" s="1"/>
+      <c r="K13" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1556,13 +1567,16 @@
         <f>SUM(B146:B157)</f>
         <v>143771</v>
       </c>
-      <c r="F14" s="7"/>
-      <c r="G14" s="8">
+      <c r="F14" s="1"/>
+      <c r="G14" s="7">
         <v>64817</v>
       </c>
-      <c r="H14" s="7"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H14" s="1"/>
+      <c r="K14" s="10">
+        <v>81629</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1576,13 +1590,19 @@
         <f>SUM(B158:B169)</f>
         <v>155890</v>
       </c>
-      <c r="F15" s="7"/>
-      <c r="G15" s="8">
+      <c r="F15" s="1"/>
+      <c r="G15" s="7">
         <v>114991</v>
       </c>
-      <c r="H15" s="9"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H15" s="8"/>
+      <c r="K15" s="10">
+        <v>81629</v>
+      </c>
+      <c r="L15">
+        <v>5909</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -1596,15 +1616,21 @@
         <f>SUM(B170:B181)</f>
         <v>174299</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="1">
         <v>80000</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="7">
         <v>157405</v>
       </c>
-      <c r="H16" s="9"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H16" s="8"/>
+      <c r="K16" s="10">
+        <v>81629</v>
+      </c>
+      <c r="L16">
+        <v>6208</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -1618,15 +1644,21 @@
         <f>SUM(B182:B193)</f>
         <v>220612</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="1">
         <v>90000</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="7">
         <v>240920</v>
       </c>
-      <c r="H17" s="10"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H17" s="9"/>
+      <c r="K17" s="10">
+        <v>582308</v>
+      </c>
+      <c r="L17">
+        <v>6985</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1640,15 +1672,21 @@
         <f>SUM(B194:B205)</f>
         <v>218775</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="1">
         <v>110000</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="7">
         <v>366887</v>
       </c>
-      <c r="H18" s="10"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H18" s="9"/>
+      <c r="K18" s="10">
+        <v>582308</v>
+      </c>
+      <c r="L18">
+        <v>6975</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -1662,15 +1700,21 @@
         <f>SUM(B206:B217)</f>
         <v>278034</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="1">
         <v>260000</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="7">
         <v>615072</v>
       </c>
-      <c r="H19" s="10"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H19" s="9"/>
+      <c r="K19" s="10">
+        <v>582308</v>
+      </c>
+      <c r="L19">
+        <v>13253</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -1684,15 +1728,21 @@
         <f>SUM(B218:B229)</f>
         <v>326382</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="1">
         <v>650000</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="7">
         <v>641419</v>
       </c>
-      <c r="H20" s="10"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H20" s="9"/>
+      <c r="K20" s="10">
+        <v>582308</v>
+      </c>
+      <c r="L20">
+        <v>25244</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -1702,15 +1752,18 @@
       <c r="D21">
         <v>2006</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="1">
         <v>850000</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="7">
         <v>585584</v>
       </c>
-      <c r="H21" s="10"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H21" s="9"/>
+      <c r="K21" s="10">
+        <v>582308</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -1720,15 +1773,18 @@
       <c r="D22">
         <v>2005</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22" s="1">
         <v>720000</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="7">
         <v>524479</v>
       </c>
-      <c r="H22" s="11"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H22" s="8"/>
+      <c r="K22" s="10">
+        <v>582308</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -1738,15 +1794,18 @@
       <c r="D23">
         <v>2004</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="1">
         <v>680000</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="7">
         <v>496785</v>
       </c>
-      <c r="H23" s="9"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H23" s="8"/>
+      <c r="K23" s="10">
+        <v>582308</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -1756,15 +1815,18 @@
       <c r="D24">
         <v>2003</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="1">
         <v>650000</v>
       </c>
-      <c r="G24" s="8">
+      <c r="G24" s="7">
         <v>458683</v>
       </c>
-      <c r="H24" s="7"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H24" s="1"/>
+      <c r="K24" s="10">
+        <v>582308</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -1774,15 +1836,18 @@
       <c r="D25">
         <v>2002</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25" s="1">
         <v>520000</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="7">
         <v>416683</v>
       </c>
-      <c r="H25" s="7"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H25" s="1"/>
+      <c r="K25" s="10">
+        <v>582308</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
@@ -1792,15 +1857,18 @@
       <c r="D26">
         <v>2001</v>
       </c>
-      <c r="F26" s="7">
+      <c r="F26" s="1">
         <v>500000</v>
       </c>
-      <c r="G26" s="8">
+      <c r="G26" s="7">
         <v>365663</v>
       </c>
-      <c r="H26" s="7"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H26" s="1"/>
+      <c r="K26" s="10">
+        <v>582308</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>26</v>
       </c>
@@ -1810,15 +1878,18 @@
       <c r="D27">
         <v>2000</v>
       </c>
-      <c r="F27" s="7">
+      <c r="F27" s="1">
         <v>530000</v>
       </c>
-      <c r="G27" s="8">
+      <c r="G27" s="7">
         <v>366776</v>
       </c>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H27" s="1"/>
+      <c r="K27" s="10">
+        <v>396105</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
@@ -1828,21 +1899,24 @@
       <c r="D28">
         <v>1999</v>
       </c>
-      <c r="F28" s="7">
+      <c r="F28" s="1">
         <v>510000</v>
       </c>
-      <c r="G28" s="8">
+      <c r="G28" s="7">
         <v>321177</v>
       </c>
-      <c r="H28" s="7"/>
-      <c r="L28" t="s">
-        <v>234</v>
-      </c>
-      <c r="M28" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H28" s="1"/>
+      <c r="K28" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N28" t="s">
+        <v>223</v>
+      </c>
+      <c r="O28" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
@@ -1852,21 +1926,24 @@
       <c r="D29">
         <v>1998</v>
       </c>
-      <c r="F29" s="7">
+      <c r="F29" s="1">
         <v>440000</v>
       </c>
-      <c r="G29" s="8">
+      <c r="G29" s="7">
         <v>275596</v>
       </c>
-      <c r="H29" s="7"/>
-      <c r="L29" t="s">
-        <v>233</v>
-      </c>
-      <c r="M29" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H29" s="1"/>
+      <c r="K29" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N29" t="s">
+        <v>222</v>
+      </c>
+      <c r="O29" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
@@ -1876,21 +1953,24 @@
       <c r="D30">
         <v>1997</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="1">
         <v>350000</v>
       </c>
-      <c r="G30" s="8">
+      <c r="G30" s="7">
         <v>272336</v>
       </c>
-      <c r="H30" s="7"/>
-      <c r="L30" t="s">
-        <v>236</v>
-      </c>
-      <c r="M30" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H30" s="1"/>
+      <c r="K30" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N30" t="s">
+        <v>225</v>
+      </c>
+      <c r="O30" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
@@ -1900,19 +1980,22 @@
       <c r="D31">
         <v>1996</v>
       </c>
-      <c r="F31" s="7"/>
-      <c r="G31" s="8">
+      <c r="F31" s="1"/>
+      <c r="G31" s="7">
         <v>253378</v>
       </c>
-      <c r="H31" s="7"/>
-      <c r="L31" t="s">
-        <v>240</v>
-      </c>
-      <c r="M31" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H31" s="1"/>
+      <c r="K31" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N31" t="s">
+        <v>229</v>
+      </c>
+      <c r="O31" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
@@ -1922,19 +2005,22 @@
       <c r="D32">
         <v>1995</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="8">
+      <c r="F32" s="1"/>
+      <c r="G32" s="7">
         <v>242122</v>
       </c>
-      <c r="H32" s="7"/>
-      <c r="L32" t="s">
-        <v>243</v>
-      </c>
-      <c r="M32" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H32" s="1"/>
+      <c r="K32" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N32" t="s">
+        <v>232</v>
+      </c>
+      <c r="O32" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>32</v>
       </c>
@@ -1944,19 +2030,22 @@
       <c r="D33">
         <v>1994</v>
       </c>
-      <c r="F33" s="7"/>
-      <c r="G33" s="8">
+      <c r="F33" s="1"/>
+      <c r="G33" s="7">
         <v>219553</v>
       </c>
-      <c r="H33" s="7"/>
-      <c r="L33" t="s">
-        <v>246</v>
-      </c>
-      <c r="M33" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H33" s="1"/>
+      <c r="K33" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N33" t="s">
+        <v>235</v>
+      </c>
+      <c r="O33" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>33</v>
       </c>
@@ -1966,13 +2055,22 @@
       <c r="D34">
         <v>1993</v>
       </c>
-      <c r="F34" s="7"/>
-      <c r="G34" s="8">
+      <c r="F34" s="1"/>
+      <c r="G34" s="7">
         <v>205404</v>
       </c>
-      <c r="H34" s="7"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H34" s="1"/>
+      <c r="K34" s="10">
+        <v>396105</v>
+      </c>
+      <c r="N34" t="s">
+        <v>238</v>
+      </c>
+      <c r="O34" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>34</v>
       </c>
@@ -1982,13 +2080,16 @@
       <c r="D35">
         <v>1992</v>
       </c>
-      <c r="F35" s="7"/>
-      <c r="G35" s="8">
+      <c r="F35" s="1"/>
+      <c r="G35" s="7">
         <v>205893</v>
       </c>
-      <c r="H35" s="7"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H35" s="1"/>
+      <c r="K35" s="10">
+        <v>396105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>35</v>
       </c>
@@ -2001,8 +2102,11 @@
       <c r="I36">
         <v>250000</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K36" s="10">
+        <v>396105</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
@@ -2015,8 +2119,11 @@
       <c r="I37">
         <v>250000</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K37" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
@@ -2029,8 +2136,11 @@
       <c r="I38">
         <v>250000</v>
       </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K38" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
@@ -2043,8 +2153,11 @@
       <c r="I39">
         <v>250000</v>
       </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K39" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
@@ -2057,8 +2170,11 @@
       <c r="I40">
         <v>250000</v>
       </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K40" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
@@ -2071,8 +2187,11 @@
       <c r="I41">
         <v>250000</v>
       </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K41" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
@@ -2085,8 +2204,11 @@
       <c r="I42">
         <v>250000</v>
       </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K42" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
@@ -2099,8 +2221,12 @@
       <c r="I43">
         <v>250000</v>
       </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K43" s="10">
+        <v>342045</v>
+      </c>
+      <c r="M43" s="10"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
@@ -2113,8 +2239,11 @@
       <c r="I44">
         <v>250000</v>
       </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K44" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
@@ -2127,8 +2256,11 @@
       <c r="I45">
         <v>250000</v>
       </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K45" s="10">
+        <v>342045</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
@@ -2141,8 +2273,12 @@
       <c r="I46">
         <v>400000</v>
       </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K46" s="10">
+        <v>342045</v>
+      </c>
+      <c r="M46" s="10"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
@@ -2155,8 +2291,12 @@
       <c r="I47">
         <v>400000</v>
       </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="K47" s="10">
+        <v>498702</v>
+      </c>
+      <c r="M47" s="10"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
@@ -2166,16 +2306,20 @@
       <c r="D48">
         <v>1979</v>
       </c>
-      <c r="F48" s="7"/>
-      <c r="G48" s="7"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
       <c r="H48">
         <v>367083</v>
       </c>
       <c r="I48">
         <v>400000</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K48" s="10">
+        <v>498702</v>
+      </c>
+      <c r="M48" s="10"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
@@ -2191,8 +2335,13 @@
       <c r="I49">
         <v>400000</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K49" s="10">
+        <v>498702</v>
+      </c>
+      <c r="M49" s="10"/>
+      <c r="N49" s="10"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>49</v>
       </c>
@@ -2208,8 +2357,12 @@
       <c r="I50">
         <v>400000</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K50" s="10">
+        <v>498702</v>
+      </c>
+      <c r="M50" s="10"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>50</v>
       </c>
@@ -2225,8 +2378,12 @@
       <c r="I51">
         <v>400000</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K51" s="10">
+        <v>498702</v>
+      </c>
+      <c r="M51" s="10"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>51</v>
       </c>
@@ -2242,8 +2399,12 @@
       <c r="I52">
         <v>400000</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K52" s="10">
+        <v>498702</v>
+      </c>
+      <c r="M52" s="10"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>52</v>
       </c>
@@ -2259,8 +2420,11 @@
       <c r="I53">
         <v>400000</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K53" s="10">
+        <v>498702</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>53</v>
       </c>
@@ -2276,8 +2440,11 @@
       <c r="I54">
         <v>400000</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K54" s="10">
+        <v>498702</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>54</v>
       </c>
@@ -2293,8 +2460,11 @@
       <c r="I55">
         <v>400000</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K55" s="10">
+        <v>498702</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>55</v>
       </c>
@@ -2310,8 +2480,11 @@
       <c r="I56">
         <v>400000</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K56" s="10">
+        <v>498702</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>56</v>
       </c>
@@ -2324,260 +2497,299 @@
       <c r="H57">
         <v>349995</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A58" s="4" t="s">
+      <c r="K57" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D58">
+        <v>1969</v>
+      </c>
+      <c r="K58" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D59">
+        <v>1968</v>
+      </c>
+      <c r="K59" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D60">
+        <v>1967</v>
+      </c>
+      <c r="K60" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D61">
+        <v>1966</v>
+      </c>
+      <c r="K61" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D62">
+        <v>1965</v>
+      </c>
+      <c r="K62" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D63">
+        <v>1964</v>
+      </c>
+      <c r="K63" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="D64">
+        <v>1963</v>
+      </c>
+      <c r="K64" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D65">
+        <v>1962</v>
+      </c>
+      <c r="K65" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D66">
+        <v>1961</v>
+      </c>
+      <c r="K66" s="10">
+        <v>383391</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D67">
+        <v>1960</v>
+      </c>
+      <c r="J67">
+        <v>128000</v>
+      </c>
+      <c r="K67" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D68">
+        <v>1959</v>
+      </c>
+      <c r="J68">
+        <v>114000</v>
+      </c>
+      <c r="K68" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B58" s="5">
+      <c r="B69" s="5">
         <v>8501</v>
       </c>
-      <c r="D58">
-        <v>1960</v>
-      </c>
-      <c r="J58">
-        <v>128000</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" s="4" t="s">
+      <c r="D69">
+        <v>1958</v>
+      </c>
+      <c r="J69">
+        <v>101000</v>
+      </c>
+      <c r="K69" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A70" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B59" s="5">
+      <c r="B70" s="5">
         <v>9949</v>
       </c>
-      <c r="D59">
-        <v>1959</v>
-      </c>
-      <c r="J59">
-        <v>114000</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" s="4" t="s">
+      <c r="D70">
+        <v>1957</v>
+      </c>
+      <c r="J70">
+        <v>98000</v>
+      </c>
+      <c r="K70" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A71" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B60" s="5">
+      <c r="B71" s="5">
         <v>10002</v>
       </c>
-      <c r="D60">
-        <v>1958</v>
-      </c>
-      <c r="J60">
-        <v>101000</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A61" s="4" t="s">
+      <c r="D71">
+        <v>1956</v>
+      </c>
+      <c r="J71">
+        <v>121800</v>
+      </c>
+      <c r="K71" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A72" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B61" s="5">
+      <c r="B72" s="5">
         <v>8525</v>
       </c>
-      <c r="D61">
-        <v>1957</v>
-      </c>
-      <c r="J61">
-        <v>98000</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A62" s="2" t="s">
+      <c r="D72">
+        <v>1955</v>
+      </c>
+      <c r="J72">
+        <v>112200</v>
+      </c>
+      <c r="K72" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B62" s="3">
+      <c r="B73" s="3">
         <v>7310</v>
       </c>
-      <c r="D62">
-        <v>1956</v>
-      </c>
-      <c r="J62">
-        <v>121800</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A63" s="2" t="s">
+      <c r="D73">
+        <v>1954</v>
+      </c>
+      <c r="J73">
+        <v>87200</v>
+      </c>
+      <c r="K73" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B63" s="3">
+      <c r="B74" s="3">
         <v>7924</v>
       </c>
-      <c r="D63">
-        <v>1955</v>
-      </c>
-      <c r="J63">
-        <v>112200</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A64" s="2" t="s">
+      <c r="D74">
+        <v>1953</v>
+      </c>
+      <c r="J74">
+        <v>67200</v>
+      </c>
+      <c r="K74" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B64" s="3">
+      <c r="B75" s="3">
         <v>7682</v>
       </c>
-      <c r="D64">
-        <v>1954</v>
-      </c>
-      <c r="J64">
-        <v>87200</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A65" s="2" t="s">
+      <c r="D75">
+        <v>1952</v>
+      </c>
+      <c r="J75">
+        <v>63300</v>
+      </c>
+      <c r="K75" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B65" s="3">
+      <c r="B76" s="3">
         <v>8404</v>
       </c>
-      <c r="D65">
-        <v>1953</v>
-      </c>
-      <c r="J65">
-        <v>67200</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A66" s="2" t="s">
+      <c r="D76">
+        <v>1951</v>
+      </c>
+      <c r="J76">
+        <v>56500</v>
+      </c>
+      <c r="K76" s="10">
+        <v>159303</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B66" s="3">
+      <c r="B77" s="3">
         <v>6818</v>
       </c>
-      <c r="D66">
-        <v>1952</v>
-      </c>
-      <c r="J66">
-        <v>63300</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A67" s="2" t="s">
+      <c r="D77">
+        <v>1950</v>
+      </c>
+      <c r="J77">
+        <v>53400</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="3">
+      <c r="B78" s="3">
         <v>6783</v>
       </c>
-      <c r="D67">
-        <v>1951</v>
-      </c>
-      <c r="J67">
-        <v>56500</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A68" s="2" t="s">
+      <c r="D78" s="10">
+        <v>1945</v>
+      </c>
+      <c r="K78" s="10">
+        <v>79293</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B68" s="3">
+      <c r="B79" s="3">
         <v>5474</v>
       </c>
-      <c r="D68">
-        <v>1950</v>
-      </c>
-      <c r="J68">
-        <v>53400</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A69" s="2" t="s">
+      <c r="D79" s="10">
+        <v>1930</v>
+      </c>
+      <c r="K79" s="10">
+        <v>55554</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A80" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="B69" s="3">
-        <v>4277</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A70" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="B70" s="3">
-        <v>4676</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B71" s="3">
-        <v>6650</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A72" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B72" s="3">
-        <v>9116</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A73" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B73" s="3">
-        <v>8447</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A74" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B74" s="5">
-        <v>6557</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A75" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B75" s="5">
-        <v>7701</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A76" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B76" s="5">
-        <v>8103</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A77" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B77" s="5">
-        <v>6490</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A78" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B78" s="5">
-        <v>6359</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A79" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B79" s="5">
-        <v>8588</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A80" s="4" t="s">
-        <v>79</v>
       </c>
       <c r="B80" s="5">
         <v>7192</v>
       </c>
+      <c r="D80" s="10">
+        <v>1910</v>
+      </c>
+      <c r="K80" s="10">
+        <v>69654</v>
+      </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="B81" s="5">
         <v>8327</v>
@@ -2585,7 +2797,7 @@
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="B82" s="5">
         <v>7560</v>
@@ -2593,7 +2805,7 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="B83" s="5">
         <v>7996</v>
@@ -2601,7 +2813,7 @@
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="B84" s="5">
         <v>8770</v>
@@ -2609,7 +2821,7 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="B85" s="5">
         <v>9303</v>
@@ -2617,7 +2829,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="B86" s="3">
         <v>6145</v>
@@ -2625,7 +2837,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="B87" s="3">
         <v>7961</v>
@@ -2633,7 +2845,7 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="B88" s="3">
         <v>7935</v>
@@ -2641,7 +2853,7 @@
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B89" s="3">
         <v>8041</v>
@@ -2649,7 +2861,7 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="B90" s="3">
         <v>8136</v>
@@ -2657,7 +2869,7 @@
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B91" s="3">
         <v>7613</v>
@@ -2665,7 +2877,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="B92" s="3">
         <v>7814</v>
@@ -2673,7 +2885,7 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B93" s="3">
         <v>8236</v>
@@ -2681,7 +2893,7 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B94" s="3">
         <v>7025</v>
@@ -2689,7 +2901,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="B95" s="3">
         <v>7023</v>
@@ -2697,7 +2909,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B96" s="3">
         <v>7457</v>
@@ -2705,7 +2917,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="B97" s="3">
         <v>8330</v>
@@ -2713,7 +2925,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B98" s="5">
         <v>5794</v>
@@ -2721,7 +2933,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="B99" s="5">
         <v>7453</v>
@@ -2729,7 +2941,7 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="B100" s="5">
         <v>6914</v>
@@ -2737,7 +2949,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="B101" s="5">
         <v>7299</v>
@@ -2745,7 +2957,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B102" s="5">
         <v>7457</v>
@@ -2753,7 +2965,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B103" s="5">
         <v>6981</v>
@@ -2761,7 +2973,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="B104" s="5">
         <v>7706</v>
@@ -2769,7 +2981,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B105" s="5">
         <v>7602</v>
@@ -2777,7 +2989,7 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B106" s="5">
         <v>5494</v>
@@ -2785,7 +2997,7 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B107" s="5">
         <v>7384</v>
@@ -2793,7 +3005,7 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="B108" s="5">
         <v>6459</v>
@@ -2801,7 +3013,7 @@
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="B109" s="5">
         <v>6697</v>
@@ -2809,7 +3021,7 @@
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B110" s="3">
         <v>5168</v>
@@ -2817,7 +3029,7 @@
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="B111" s="3">
         <v>5762</v>
@@ -2825,7 +3037,7 @@
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" s="2" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="B112" s="3">
         <v>5349</v>
@@ -2833,7 +3045,7 @@
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B113" s="3">
         <v>5992</v>
@@ -2841,7 +3053,7 @@
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="B114" s="3">
         <v>6099</v>
@@ -2849,7 +3061,7 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="B115" s="3">
         <v>6037</v>
@@ -2857,7 +3069,7 @@
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B116" s="3">
         <v>6592</v>
@@ -2865,7 +3077,7 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B117" s="3">
         <v>6867</v>
@@ -2873,7 +3085,7 @@
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="B118" s="3">
         <v>7131</v>
@@ -2881,7 +3093,7 @@
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="B119" s="3">
         <v>6075</v>
@@ -2889,7 +3101,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="B120" s="3">
         <v>7690</v>
@@ -2897,7 +3109,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="B121" s="3">
         <v>6372</v>
@@ -2905,7 +3117,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="B122" s="5">
         <v>5549</v>
@@ -2913,7 +3125,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="B123" s="5">
         <v>5438</v>
@@ -2921,7 +3133,7 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="B124" s="5">
         <v>5381</v>
@@ -2929,7 +3141,7 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="B125" s="5">
         <v>6091</v>
@@ -2937,7 +3149,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="B126" s="5">
         <v>5925</v>
@@ -2945,7 +3157,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="B127" s="5">
         <v>6415</v>
@@ -2953,7 +3165,7 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B128" s="5">
         <v>6454</v>
@@ -2961,7 +3173,7 @@
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="B129" s="5">
         <v>6252</v>
@@ -2969,7 +3181,7 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="B130" s="5">
         <v>6097</v>
@@ -2977,7 +3189,7 @@
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="B131" s="5">
         <v>6594</v>
@@ -2985,7 +3197,7 @@
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="B132" s="5">
         <v>7846</v>
@@ -2993,7 +3205,7 @@
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="B133" s="5">
         <v>8912</v>
@@ -3001,7 +3213,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="B134" s="3">
         <v>7153</v>
@@ -3009,7 +3221,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="B135" s="3">
         <v>7543</v>
@@ -3017,7 +3229,7 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="B136" s="3">
         <v>8089</v>
@@ -3025,7 +3237,7 @@
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="B137" s="3">
         <v>8890</v>
@@ -3033,7 +3245,7 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="B138" s="3">
         <v>8082</v>
@@ -3041,7 +3253,7 @@
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="B139" s="3">
         <v>10333</v>
@@ -3049,7 +3261,7 @@
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="B140" s="3">
         <v>9561</v>
@@ -3057,7 +3269,7 @@
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="B141" s="3">
         <v>10619</v>
@@ -3065,7 +3277,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="B142" s="3">
         <v>10445</v>
@@ -3073,7 +3285,7 @@
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="B143" s="3">
         <v>11156</v>
@@ -3081,7 +3293,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="B144" s="3">
         <v>11345</v>
@@ -3089,7 +3301,7 @@
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="B145" s="3">
         <v>14303</v>
@@ -3097,7 +3309,7 @@
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="B146" s="5">
         <v>10815</v>
@@ -3105,7 +3317,7 @@
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="B147" s="5">
         <v>9787</v>
@@ -3113,7 +3325,7 @@
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A148" s="4" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="B148" s="5">
         <v>9903</v>
@@ -3121,7 +3333,7 @@
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="B149" s="5">
         <v>10605</v>
@@ -3129,7 +3341,7 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A150" s="4" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="B150" s="5">
         <v>10398</v>
@@ -3137,7 +3349,7 @@
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A151" s="4" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="B151" s="5">
         <v>11321</v>
@@ -3145,7 +3357,7 @@
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A152" s="4" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="B152" s="5">
         <v>10125</v>
@@ -3153,7 +3365,7 @@
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A153" s="4" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="B153" s="5">
         <v>11817</v>
@@ -3161,7 +3373,7 @@
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="B154" s="5">
         <v>10087</v>
@@ -3169,7 +3381,7 @@
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A155" s="4" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="B155" s="5">
         <v>10422</v>
@@ -3177,7 +3389,7 @@
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A156" s="4" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="B156" s="5">
         <v>18451</v>
@@ -3185,7 +3397,7 @@
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B157" s="5">
         <v>20040</v>
@@ -3193,7 +3405,7 @@
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="B158" s="3">
         <v>11143</v>
@@ -3201,7 +3413,7 @@
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="B159" s="3">
         <v>12604</v>
@@ -3209,7 +3421,7 @@
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="B160" s="3">
         <v>12224</v>
@@ -3217,7 +3429,7 @@
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="B161" s="3">
         <v>12828</v>
@@ -3225,7 +3437,7 @@
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="B162" s="3">
         <v>13960</v>
@@ -3233,7 +3445,7 @@
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="B163" s="3">
         <v>12881</v>
@@ -3241,7 +3453,7 @@
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A164" s="2" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="B164" s="3">
         <v>11936</v>
@@ -3249,7 +3461,7 @@
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A165" s="2" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="B165" s="3">
         <v>12892</v>
@@ -3257,7 +3469,7 @@
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A166" s="2" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="B166" s="3">
         <v>9728</v>
@@ -3265,7 +3477,7 @@
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A167" s="2" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="B167" s="3">
         <v>11972</v>
@@ -3273,7 +3485,7 @@
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A168" s="2" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="B168" s="3">
         <v>15898</v>
@@ -3281,7 +3493,7 @@
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A169" s="2" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="B169" s="3">
         <v>17824</v>
@@ -3289,7 +3501,7 @@
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A170" s="4" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="B170" s="5">
         <v>10877</v>
@@ -3297,7 +3509,7 @@
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A171" s="4" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="B171" s="5">
         <v>13461</v>
@@ -3305,7 +3517,7 @@
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A172" s="4" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="B172" s="5">
         <v>10851</v>
@@ -3313,7 +3525,7 @@
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A173" s="4" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="B173" s="5">
         <v>12750</v>
@@ -3321,7 +3533,7 @@
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A174" s="4" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="B174" s="5">
         <v>13105</v>
@@ -3329,7 +3541,7 @@
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A175" s="4" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="B175" s="5">
         <v>13313</v>
@@ -3337,7 +3549,7 @@
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" s="4" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="B176" s="5">
         <v>13811</v>
@@ -3345,7 +3557,7 @@
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A177" s="4" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="B177" s="5">
         <v>14612</v>
@@ -3353,7 +3565,7 @@
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A178" s="4" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="B178" s="5">
         <v>11340</v>
@@ -3361,7 +3573,7 @@
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A179" s="4" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="B179" s="5">
         <v>16119</v>
@@ -3369,7 +3581,7 @@
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A180" s="4" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="B180" s="5">
         <v>22384</v>
@@ -3377,7 +3589,7 @@
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A181" s="4" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="B181" s="5">
         <v>21676</v>
@@ -3385,7 +3597,7 @@
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A182" s="2" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="B182" s="3">
         <v>15589</v>
@@ -3393,7 +3605,7 @@
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A183" s="2" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="B183" s="3">
         <v>15509</v>
@@ -3401,7 +3613,7 @@
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A184" s="2" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="B184" s="3">
         <v>13360</v>
@@ -3409,7 +3621,7 @@
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A185" s="2" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="B185" s="3">
         <v>18155</v>
@@ -3417,7 +3629,7 @@
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A186" s="2" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="B186" s="3">
         <v>23009</v>
@@ -3425,7 +3637,7 @@
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A187" s="2" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="B187" s="3">
         <v>22529</v>
@@ -3433,7 +3645,7 @@
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A188" s="2" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="B188" s="3">
         <v>17721</v>
@@ -3441,7 +3653,7 @@
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A189" s="2" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="B189" s="3">
         <v>18983</v>
@@ -3449,7 +3661,7 @@
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A190" s="2" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="B190" s="3">
         <v>16967</v>
@@ -3457,7 +3669,7 @@
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A191" s="2" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="B191" s="3">
         <v>18440</v>
@@ -3465,7 +3677,7 @@
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A192" s="2" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="B192" s="3">
         <v>21341</v>
@@ -3473,7 +3685,7 @@
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A193" s="2" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="B193" s="3">
         <v>19009</v>
@@ -3481,7 +3693,7 @@
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A194" s="4" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="B194" s="5">
         <v>16454</v>
@@ -3489,7 +3701,7 @@
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A195" s="4" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="B195" s="5">
         <v>18070</v>
@@ -3497,7 +3709,7 @@
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A196" s="4" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="B196" s="5">
         <v>16488</v>
@@ -3505,7 +3717,7 @@
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A197" s="4" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="B197" s="5">
         <v>20076</v>
@@ -3513,7 +3725,7 @@
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A198" s="4" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="B198" s="5">
         <v>18494</v>
@@ -3521,7 +3733,7 @@
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A199" s="4" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="B199" s="5">
         <v>19487</v>
@@ -3529,7 +3741,7 @@
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A200" s="4" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="B200" s="5">
         <v>18343</v>
@@ -3537,7 +3749,7 @@
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A201" s="4" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="B201" s="5">
         <v>17537</v>
@@ -3545,7 +3757,7 @@
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A202" s="4" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="B202" s="5">
         <v>15540</v>
@@ -3553,7 +3765,7 @@
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A203" s="4" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="B203" s="5">
         <v>19111</v>
@@ -3561,7 +3773,7 @@
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A204" s="4" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="B204" s="5">
         <v>18682</v>
@@ -3569,7 +3781,7 @@
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A205" s="4" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="B205" s="5">
         <v>20493</v>
@@ -3577,7 +3789,7 @@
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A206" s="2" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="B206" s="3">
         <v>17443</v>
@@ -3585,7 +3797,7 @@
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A207" s="2" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="B207" s="3">
         <v>19153</v>
@@ -3593,7 +3805,7 @@
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A208" s="2" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="B208" s="3">
         <v>23315</v>
@@ -3601,7 +3813,7 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A209" s="2" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="B209" s="3">
         <v>25011</v>
@@ -3609,7 +3821,7 @@
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A210" s="2" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="B210" s="3">
         <v>19858</v>
@@ -3617,7 +3829,7 @@
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A211" s="2" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="B211" s="3">
         <v>22618</v>
@@ -3625,7 +3837,7 @@
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A212" s="2" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="B212" s="3">
         <v>22510</v>
@@ -3633,7 +3845,7 @@
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A213" s="2" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="B213" s="3">
         <v>24392</v>
@@ -3641,7 +3853,7 @@
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A214" s="2" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="B214" s="3">
         <v>26693</v>
@@ -3649,7 +3861,7 @@
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A215" s="2" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="B215" s="3">
         <v>22133</v>
@@ -3657,7 +3869,7 @@
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A216" s="2" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="B216" s="3">
         <v>25952</v>
@@ -3665,7 +3877,7 @@
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A217" s="2" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="B217" s="3">
         <v>28956</v>
@@ -3673,7 +3885,7 @@
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A218" s="4" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="B218" s="5">
         <v>19921</v>
@@ -3681,7 +3893,7 @@
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A219" s="4" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="B219" s="5">
         <v>24245</v>
@@ -3689,7 +3901,7 @@
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A220" s="4" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="B220" s="5">
         <v>25492</v>
@@ -3697,7 +3909,7 @@
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A221" s="4" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="B221" s="5">
         <v>27658</v>
@@ -3705,7 +3917,7 @@
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A222" s="4" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="B222" s="5">
         <v>25437</v>
@@ -3713,7 +3925,7 @@
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A223" s="4" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="B223" s="5">
         <v>26816</v>
@@ -3721,7 +3933,7 @@
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A224" s="4" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="B224" s="5">
         <v>27263</v>
@@ -3729,7 +3941,7 @@
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A225" s="4" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="B225" s="5">
         <v>31334</v>
@@ -3737,7 +3949,7 @@
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A226" s="4" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="B226" s="5">
         <v>24549</v>
@@ -3745,7 +3957,7 @@
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A227" s="4" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="B227" s="5">
         <v>30403</v>
@@ -3753,7 +3965,7 @@
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A228" s="4" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="B228" s="5">
         <v>29784</v>
@@ -3761,7 +3973,7 @@
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A229" s="4" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="B229" s="5">
         <v>33480</v>

</xml_diff>

<commit_message>
cleanup, floor area, materials and emissions
</commit_message>
<xml_diff>
--- a/inflow_validation.xlsx
+++ b/inflow_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marita/Documents/GitHub/MFA2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC3C3D92-751A-7C48-8F1A-EF8448178246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37A7896-C475-9646-8316-475F3BC93112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tabla-6150" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="242">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -753,6 +753,12 @@
   </si>
   <si>
     <t>demolition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">demolition </t>
+  </si>
+  <si>
+    <t>https://ec.europa.eu/environment/pdf/waste/studies/deliverables/CDW_Spain_Factsheet_Final.pdf</t>
   </si>
 </sst>
 </file>
@@ -2088,6 +2094,12 @@
       <c r="K35" s="10">
         <v>396105</v>
       </c>
+      <c r="N35" t="s">
+        <v>240</v>
+      </c>
+      <c r="O35" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">

</xml_diff>